<commit_message>
Auto: 2026-09-28 scrape results
</commit_message>
<xml_diff>
--- a/results/auto_Cape_Town_Animal_Welfare_from_master.xlsx
+++ b/results/auto_Cape_Town_Animal_Welfare_from_master.xlsx
@@ -14,7 +14,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="19" uniqueCount="15">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="20" uniqueCount="16">
   <si>
     <t>Organisation Name</t>
   </si>
@@ -59,6 +59,9 @@
   </si>
   <si>
     <t>aro@animalrescue.org.za</t>
+  </si>
+  <si>
+    <t>Yes</t>
   </si>
 </sst>
 </file>
@@ -429,6 +432,9 @@
       <c r="D2" t="s">
         <v>12</v>
       </c>
+      <c r="G2" t="s">
+        <v>15</v>
+      </c>
     </row>
     <row r="3" spans="1:7">
       <c r="A3" t="s">

</xml_diff>